<commit_message>
Forms sync auto batch 9: 3847 files
</commit_message>
<xml_diff>
--- a/survey_templates/043_political_liberalism_assessment--survey_templates.xlsx
+++ b/survey_templates/043_political_liberalism_assessment--survey_templates.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1102,8 +1102,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1131,12 +1131,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>option1</t>
+          <t>option_1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>option1</t>
+          <t>Option 1</t>
         </is>
       </c>
     </row>
@@ -1148,12 +1148,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>option2</t>
+          <t>option_2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>option2</t>
+          <t>Option 2</t>
         </is>
       </c>
     </row>
@@ -1165,12 +1165,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>option3</t>
+          <t>option_3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>option3</t>
+          <t>Option 3</t>
         </is>
       </c>
     </row>
@@ -1182,12 +1182,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>option1</t>
+          <t>option_1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>option1</t>
+          <t>Option 1</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1199,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>option2</t>
+          <t>option_2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>option2</t>
+          <t>Option 2</t>
         </is>
       </c>
     </row>
@@ -1216,12 +1216,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>option3</t>
+          <t>option_3</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>option3</t>
+          <t>Option 3</t>
         </is>
       </c>
     </row>
@@ -1233,12 +1233,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>option1</t>
+          <t>option_1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>option1</t>
+          <t>Option 1</t>
         </is>
       </c>
     </row>
@@ -1250,12 +1250,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>option2</t>
+          <t>option_2</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>option2</t>
+          <t>Option 2</t>
         </is>
       </c>
     </row>
@@ -1267,12 +1267,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>option3</t>
+          <t>option_3</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>option3</t>
+          <t>Option 3</t>
         </is>
       </c>
     </row>
@@ -1284,12 +1284,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>option1</t>
+          <t>option_1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>option1</t>
+          <t>Option 1</t>
         </is>
       </c>
     </row>
@@ -1301,12 +1301,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>option2</t>
+          <t>option_2</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>option2</t>
+          <t>Option 2</t>
         </is>
       </c>
     </row>
@@ -1318,12 +1318,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>option3</t>
+          <t>option_3</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>option3</t>
+          <t>Option 3</t>
         </is>
       </c>
     </row>
@@ -1335,12 +1335,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>option1</t>
+          <t>option_1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>option1</t>
+          <t>Option 1</t>
         </is>
       </c>
     </row>
@@ -1352,12 +1352,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>option2</t>
+          <t>option_2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>option2</t>
+          <t>Option 2</t>
         </is>
       </c>
     </row>
@@ -1369,12 +1369,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>option3</t>
+          <t>option_3</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>option3</t>
+          <t>Option 3</t>
         </is>
       </c>
     </row>

</xml_diff>